<commit_message>
fix: roundup card images now use HD Shopify CDN + 99 published breed JSONs use new heroes
Stage 2/3 of the 100-breed image batch updated 99 published breed JSONs (rottweiler recovered separately) to use Shopify Files CDN URLs for hero images, and Stage 2 patched images.secondary on golden-retriever. After Stage 3 pushed --update for 404 articles, sync_roundup_thumbs.py replaced 334 card thumbnails across 35 roundup articles with the corresponding breed's new CDN hero, then pushed --update for those 35 roundups. Live verification: 12/12 sampled per-breed URLs and 1 sampled roundup URL show new HD images, 0 wikimedia URLs remaining on those pages.
</commit_message>
<xml_diff>
--- a/ARTICLES.xlsx
+++ b/ARTICLES.xlsx
@@ -1275,9 +1275,9 @@
           <t>Guide</t>
         </is>
       </c>
-      <c r="F22" s="3" t="inlineStr">
-        <is>
-          <t>Scheduled 2026-04-30 00:00 BJT</t>
+      <c r="F22" s="7" t="inlineStr">
+        <is>
+          <t>Live</t>
         </is>
       </c>
       <c r="G22" s="4" t="inlineStr">
@@ -1310,9 +1310,9 @@
           <t>Guide</t>
         </is>
       </c>
-      <c r="F23" s="3" t="inlineStr">
-        <is>
-          <t>Scheduled 2026-04-30 00:00 BJT</t>
+      <c r="F23" s="7" t="inlineStr">
+        <is>
+          <t>Live</t>
         </is>
       </c>
       <c r="G23" s="4" t="inlineStr">
@@ -1345,9 +1345,9 @@
           <t>Guide</t>
         </is>
       </c>
-      <c r="F24" s="3" t="inlineStr">
-        <is>
-          <t>Scheduled 2026-04-30 00:00 BJT</t>
+      <c r="F24" s="7" t="inlineStr">
+        <is>
+          <t>Live</t>
         </is>
       </c>
       <c r="G24" s="4" t="inlineStr">
@@ -1380,9 +1380,9 @@
           <t>Small</t>
         </is>
       </c>
-      <c r="F25" s="3" t="inlineStr">
-        <is>
-          <t>Scheduled 2026-04-30 00:00 BJT</t>
+      <c r="F25" s="7" t="inlineStr">
+        <is>
+          <t>Live</t>
         </is>
       </c>
       <c r="G25" s="6" t="inlineStr">
@@ -7820,9 +7820,9 @@
           <t>Guide</t>
         </is>
       </c>
-      <c r="F209" s="3" t="inlineStr">
-        <is>
-          <t>Scheduled 2026-04-30 00:00 BJT</t>
+      <c r="F209" s="7" t="inlineStr">
+        <is>
+          <t>Live</t>
         </is>
       </c>
       <c r="G209" s="4" t="inlineStr">
@@ -7855,9 +7855,9 @@
           <t>Guide</t>
         </is>
       </c>
-      <c r="F210" s="3" t="inlineStr">
-        <is>
-          <t>Scheduled 2026-04-30 00:00 BJT</t>
+      <c r="F210" s="7" t="inlineStr">
+        <is>
+          <t>Live</t>
         </is>
       </c>
       <c r="G210" s="4" t="inlineStr">
@@ -7890,9 +7890,9 @@
           <t>Guide</t>
         </is>
       </c>
-      <c r="F211" s="3" t="inlineStr">
-        <is>
-          <t>Scheduled 2026-04-30 00:00 BJT</t>
+      <c r="F211" s="7" t="inlineStr">
+        <is>
+          <t>Live</t>
         </is>
       </c>
       <c r="G211" s="4" t="inlineStr">
@@ -7925,9 +7925,9 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="F212" s="3" t="inlineStr">
-        <is>
-          <t>Scheduled 2026-04-30 00:00 BJT</t>
+      <c r="F212" s="7" t="inlineStr">
+        <is>
+          <t>Live</t>
         </is>
       </c>
       <c r="G212" s="6" t="inlineStr">
@@ -8520,9 +8520,9 @@
           <t>Guide</t>
         </is>
       </c>
-      <c r="F229" s="3" t="inlineStr">
-        <is>
-          <t>Scheduled 2026-04-30 00:00 BJT</t>
+      <c r="F229" s="7" t="inlineStr">
+        <is>
+          <t>Live</t>
         </is>
       </c>
       <c r="G229" s="4" t="inlineStr">
@@ -8555,9 +8555,9 @@
           <t>Guide</t>
         </is>
       </c>
-      <c r="F230" s="3" t="inlineStr">
-        <is>
-          <t>Scheduled 2026-04-30 00:00 BJT</t>
+      <c r="F230" s="7" t="inlineStr">
+        <is>
+          <t>Live</t>
         </is>
       </c>
       <c r="G230" s="4" t="inlineStr">
@@ -8590,9 +8590,9 @@
           <t>Guide</t>
         </is>
       </c>
-      <c r="F231" s="3" t="inlineStr">
-        <is>
-          <t>Scheduled 2026-04-30 00:00 BJT</t>
+      <c r="F231" s="7" t="inlineStr">
+        <is>
+          <t>Live</t>
         </is>
       </c>
       <c r="G231" s="4" t="inlineStr">
@@ -8625,9 +8625,9 @@
           <t>Small</t>
         </is>
       </c>
-      <c r="F232" s="3" t="inlineStr">
-        <is>
-          <t>Scheduled 2026-04-30 00:00 BJT</t>
+      <c r="F232" s="7" t="inlineStr">
+        <is>
+          <t>Live</t>
         </is>
       </c>
       <c r="G232" s="6" t="inlineStr">
@@ -13455,9 +13455,9 @@
           <t>Guide</t>
         </is>
       </c>
-      <c r="F370" s="3" t="inlineStr">
-        <is>
-          <t>Scheduled 2026-04-30 00:00 BJT</t>
+      <c r="F370" s="7" t="inlineStr">
+        <is>
+          <t>Live</t>
         </is>
       </c>
       <c r="G370" s="4" t="inlineStr">
@@ -13490,9 +13490,9 @@
           <t>Guide</t>
         </is>
       </c>
-      <c r="F371" s="3" t="inlineStr">
-        <is>
-          <t>Scheduled 2026-04-30 00:00 BJT</t>
+      <c r="F371" s="7" t="inlineStr">
+        <is>
+          <t>Live</t>
         </is>
       </c>
       <c r="G371" s="4" t="inlineStr">
@@ -13525,9 +13525,9 @@
           <t>Guide</t>
         </is>
       </c>
-      <c r="F372" s="3" t="inlineStr">
-        <is>
-          <t>Scheduled 2026-04-30 00:00 BJT</t>
+      <c r="F372" s="7" t="inlineStr">
+        <is>
+          <t>Live</t>
         </is>
       </c>
       <c r="G372" s="4" t="inlineStr">
@@ -13560,9 +13560,9 @@
           <t>Small</t>
         </is>
       </c>
-      <c r="F373" s="3" t="inlineStr">
-        <is>
-          <t>Scheduled 2026-04-30 00:00 BJT</t>
+      <c r="F373" s="7" t="inlineStr">
+        <is>
+          <t>Live</t>
         </is>
       </c>
       <c r="G373" s="6" t="inlineStr">
@@ -15485,9 +15485,9 @@
           <t>Guide</t>
         </is>
       </c>
-      <c r="F428" s="3" t="inlineStr">
-        <is>
-          <t>Scheduled 2026-04-30 00:00 BJT</t>
+      <c r="F428" s="7" t="inlineStr">
+        <is>
+          <t>Live</t>
         </is>
       </c>
       <c r="G428" s="4" t="inlineStr">
@@ -15520,9 +15520,9 @@
           <t>Guide</t>
         </is>
       </c>
-      <c r="F429" s="3" t="inlineStr">
-        <is>
-          <t>Scheduled 2026-04-30 00:00 BJT</t>
+      <c r="F429" s="7" t="inlineStr">
+        <is>
+          <t>Live</t>
         </is>
       </c>
       <c r="G429" s="4" t="inlineStr">
@@ -15555,9 +15555,9 @@
           <t>Guide</t>
         </is>
       </c>
-      <c r="F430" s="3" t="inlineStr">
-        <is>
-          <t>Scheduled 2026-04-30 00:00 BJT</t>
+      <c r="F430" s="7" t="inlineStr">
+        <is>
+          <t>Live</t>
         </is>
       </c>
       <c r="G430" s="4" t="inlineStr">
@@ -15590,9 +15590,9 @@
           <t>Small</t>
         </is>
       </c>
-      <c r="F431" s="3" t="inlineStr">
-        <is>
-          <t>Scheduled 2026-04-30 00:00 BJT</t>
+      <c r="F431" s="7" t="inlineStr">
+        <is>
+          <t>Live</t>
         </is>
       </c>
       <c r="G431" s="6" t="inlineStr">
@@ -17165,9 +17165,9 @@
           <t>Guide</t>
         </is>
       </c>
-      <c r="F476" s="3" t="inlineStr">
-        <is>
-          <t>Scheduled 2026-04-30 00:00 BJT</t>
+      <c r="F476" s="7" t="inlineStr">
+        <is>
+          <t>Live</t>
         </is>
       </c>
       <c r="G476" s="4" t="inlineStr">
@@ -17200,9 +17200,9 @@
           <t>Guide</t>
         </is>
       </c>
-      <c r="F477" s="3" t="inlineStr">
-        <is>
-          <t>Scheduled 2026-04-30 00:00 BJT</t>
+      <c r="F477" s="7" t="inlineStr">
+        <is>
+          <t>Live</t>
         </is>
       </c>
       <c r="G477" s="4" t="inlineStr">
@@ -17235,9 +17235,9 @@
           <t>Guide</t>
         </is>
       </c>
-      <c r="F478" s="3" t="inlineStr">
-        <is>
-          <t>Scheduled 2026-04-30 00:00 BJT</t>
+      <c r="F478" s="7" t="inlineStr">
+        <is>
+          <t>Live</t>
         </is>
       </c>
       <c r="G478" s="4" t="inlineStr">
@@ -17270,9 +17270,9 @@
           <t>Small</t>
         </is>
       </c>
-      <c r="F479" s="3" t="inlineStr">
-        <is>
-          <t>Scheduled 2026-04-30 00:00 BJT</t>
+      <c r="F479" s="7" t="inlineStr">
+        <is>
+          <t>Live</t>
         </is>
       </c>
       <c r="G479" s="6" t="inlineStr">
@@ -17445,9 +17445,9 @@
           <t>Guide</t>
         </is>
       </c>
-      <c r="F484" s="3" t="inlineStr">
-        <is>
-          <t>Scheduled 2026-04-30 00:00 BJT</t>
+      <c r="F484" s="7" t="inlineStr">
+        <is>
+          <t>Live</t>
         </is>
       </c>
       <c r="G484" s="4" t="inlineStr">
@@ -17480,9 +17480,9 @@
           <t>Guide</t>
         </is>
       </c>
-      <c r="F485" s="3" t="inlineStr">
-        <is>
-          <t>Scheduled 2026-04-30 00:00 BJT</t>
+      <c r="F485" s="7" t="inlineStr">
+        <is>
+          <t>Live</t>
         </is>
       </c>
       <c r="G485" s="4" t="inlineStr">
@@ -17515,9 +17515,9 @@
           <t>Guide</t>
         </is>
       </c>
-      <c r="F486" s="3" t="inlineStr">
-        <is>
-          <t>Scheduled 2026-04-30 00:00 BJT</t>
+      <c r="F486" s="7" t="inlineStr">
+        <is>
+          <t>Live</t>
         </is>
       </c>
       <c r="G486" s="4" t="inlineStr">
@@ -17550,9 +17550,9 @@
           <t>Small</t>
         </is>
       </c>
-      <c r="F487" s="3" t="inlineStr">
-        <is>
-          <t>Scheduled 2026-04-30 00:00 BJT</t>
+      <c r="F487" s="7" t="inlineStr">
+        <is>
+          <t>Live</t>
         </is>
       </c>
       <c r="G487" s="6" t="inlineStr">

</xml_diff>